<commit_message>
Add Telegram bot as a second intake channel, same form/flow
Telegram Mini App form (same fields as the WhatsApp Flow) backed by
the same Google Sheets/Drive integration. No Meta-style encryption or
business verification required - just a signed initData HMAC check
per Telegram's documented Mini App auth scheme. Adds Channel and
Telegram Username columns to the shared sheet schema.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/alumni_tracer_template.xlsx
+++ b/templates/alumni_tracer_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Z1"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -423,6 +423,8 @@
     <col min="22" max="22" width="24.83203125" customWidth="1"/>
     <col min="23" max="23" width="24.83203125" customWidth="1"/>
     <col min="24" max="24" width="24.83203125" customWidth="1"/>
+    <col min="25" max="25" width="24.83203125" customWidth="1"/>
+    <col min="26" max="26" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,78 +432,84 @@
         <v>Timestamp</v>
       </c>
       <c r="B1" t="str">
+        <v>Channel</v>
+      </c>
+      <c r="C1" t="str">
         <v>Nomor WhatsApp</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
+        <v>Telegram Username</v>
+      </c>
+      <c r="E1" t="str">
         <v>Nama Lengkap</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>Alumni Program Beasiswa</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>Asal Kampus</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Tahun Masuk Beasiswa</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Jurusan</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Jenis Kelamin</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Nomor HP</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Domisili</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Provinsi</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Instagram/Facebook</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Tanggal Lulus Pendidikan dengan Beasiswa BAZNAS</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>IPK</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>Lama Kuliah (Bulan)</v>
       </c>
-      <c r="P1" t="str">
+      <c r="R1" t="str">
         <v>Masa Tunggu (Bulan)</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="S1" t="str">
         <v>Sektor Pekerjaan</v>
       </c>
-      <c r="R1" t="str">
+      <c r="T1" t="str">
         <v>Kategori Sektor</v>
       </c>
-      <c r="S1" t="str">
+      <c r="U1" t="str">
         <v>Tempat Bekerja</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>Posisi/Jabatan di Tempat Kerja</v>
       </c>
-      <c r="U1" t="str">
+      <c r="W1" t="str">
         <v>Pendapatan</v>
       </c>
-      <c r="V1" t="str">
+      <c r="X1" t="str">
         <v>Jobdesk Singkat</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Y1" t="str">
         <v>Kata-Kata Motivasi</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Z1" t="str">
         <v>Link Foto Terbaik</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>